<commit_message>
bugfixed models after sampling
</commit_message>
<xml_diff>
--- a/smoment/autopacmen_output/Mitocore_MitoMammal/Mitocore_MitoMammal_kcats_calibrated.xlsx
+++ b/smoment/autopacmen_output/Mitocore_MitoMammal/Mitocore_MitoMammal_kcats_calibrated.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>original_kcats</t>
   </si>
@@ -25,37 +25,49 @@
     <t>original_reactions</t>
   </si>
   <si>
+    <t>CIII_MitoCore_forward</t>
+  </si>
+  <si>
+    <t>PDHm_forward</t>
+  </si>
+  <si>
+    <t>PDHm_reverse</t>
+  </si>
+  <si>
+    <t>CIV_MitoCore_forward</t>
+  </si>
+  <si>
+    <t>CIV_MitoCore_reverse</t>
+  </si>
+  <si>
+    <t>ICDHxm_forward</t>
+  </si>
+  <si>
+    <t>ICDHxm_reverse</t>
+  </si>
+  <si>
+    <t>ACONTm_forward</t>
+  </si>
+  <si>
+    <t>SUCOASm_reverse</t>
+  </si>
+  <si>
+    <t>ACONT_forward</t>
+  </si>
+  <si>
+    <t>AACTOORm_MitoCore_forward</t>
+  </si>
+  <si>
+    <t>AACTOORm_MitoCore_reverse</t>
+  </si>
+  <si>
+    <t>r0074_forward</t>
+  </si>
+  <si>
+    <t>r0074_reverse</t>
+  </si>
+  <si>
     <t>CV_MitoCore_forward</t>
-  </si>
-  <si>
-    <t>CIV_MitoCore_forward</t>
-  </si>
-  <si>
-    <t>CIV_MitoCore_reverse</t>
-  </si>
-  <si>
-    <t>ACONTm_forward</t>
-  </si>
-  <si>
-    <t>PDHm_forward</t>
-  </si>
-  <si>
-    <t>PDHm_reverse</t>
-  </si>
-  <si>
-    <t>ICDHxm_forward</t>
-  </si>
-  <si>
-    <t>ICDHxm_reverse</t>
-  </si>
-  <si>
-    <t>ACONT_forward</t>
-  </si>
-  <si>
-    <t>SUCOASm_reverse</t>
-  </si>
-  <si>
-    <t>CIII_MitoCore_forward</t>
   </si>
 </sst>
 </file>
@@ -413,7 +425,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -432,10 +444,10 @@
         <v>3</v>
       </c>
       <c r="B2">
-        <v>18.5</v>
+        <v>79</v>
       </c>
       <c r="C2">
-        <v>340.2551843437593</v>
+        <v>3964.739189541615</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -443,10 +455,10 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>38.1</v>
+        <v>0.48</v>
       </c>
       <c r="C3">
-        <v>1906.50670314972</v>
+        <v>19.58879791251504</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -454,10 +466,10 @@
         <v>5</v>
       </c>
       <c r="B4">
-        <v>13.33333</v>
+        <v>0.48</v>
       </c>
       <c r="C4">
-        <v>667.193780060558</v>
+        <v>19.58879791251504</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -465,10 +477,10 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>5.2</v>
+        <v>38.85</v>
       </c>
       <c r="C5">
-        <v>260.2056066977244</v>
+        <v>1949.744769352464</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -476,10 +488,10 @@
         <v>7</v>
       </c>
       <c r="B6">
-        <v>2.4</v>
+        <v>38.85</v>
       </c>
       <c r="C6">
-        <v>119.3510831543757</v>
+        <v>1949.744769352464</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -487,10 +499,10 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <v>2.4</v>
+        <v>16.7</v>
       </c>
       <c r="C7">
-        <v>119.3510831543757</v>
+        <v>838.122184950694</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -498,10 +510,10 @@
         <v>9</v>
       </c>
       <c r="B8">
-        <v>20.5</v>
+        <v>19.7</v>
       </c>
       <c r="C8">
-        <v>1025.810664543069</v>
+        <v>988.6830564987227</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -509,10 +521,10 @@
         <v>10</v>
       </c>
       <c r="B9">
-        <v>81.685</v>
+        <v>5.2</v>
       </c>
       <c r="C9">
-        <v>4087.480201619541</v>
+        <v>260.9726593969617</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -520,10 +532,10 @@
         <v>11</v>
       </c>
       <c r="B10">
-        <v>5.2</v>
+        <v>19.8</v>
       </c>
       <c r="C10">
-        <v>260.2056446959795</v>
+        <v>993.7032181483266</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -531,10 +543,10 @@
         <v>12</v>
       </c>
       <c r="B11">
-        <v>19.8</v>
+        <v>5.2</v>
       </c>
       <c r="C11">
-        <v>990.7828903040836</v>
+        <v>260.9726206650865</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -542,10 +554,54 @@
         <v>13</v>
       </c>
       <c r="B12">
-        <v>79</v>
+        <v>0.67</v>
       </c>
       <c r="C12">
-        <v>3953.123158137042</v>
+        <v>33.62498583487577</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13">
+        <v>0.67</v>
+      </c>
+      <c r="C13">
+        <v>33.62498583487577</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14">
+        <v>1.4</v>
+      </c>
+      <c r="C14">
+        <v>70.26175022732079</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15">
+        <v>1.4</v>
+      </c>
+      <c r="C15">
+        <v>70.26175022732079</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16">
+        <v>18.5</v>
+      </c>
+      <c r="C16">
+        <v>862.8698719532498</v>
       </c>
     </row>
   </sheetData>

</xml_diff>